<commit_message>
cliquer sur les marqueurs pour échanger + màj vérifierClubDansPoule
</commit_message>
<xml_diff>
--- a/fichiers_csv/fichiers équipes/poules_senior_masculin.xlsx
+++ b/fichiers_csv/fichiers équipes/poules_senior_masculin.xlsx
@@ -4,7 +4,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Niveau 1" sheetId="1" r:id="rId1"/>
-    <sheet name="Récapitulatif" sheetId="2" r:id="rId2"/>
+    <sheet name="Niveau 2" sheetId="2" r:id="rId2"/>
+    <sheet name="Niveau 3" sheetId="3" r:id="rId3"/>
+    <sheet name="Niveau 4" sheetId="4" r:id="rId4"/>
+    <sheet name="Récapitulatif" sheetId="5" r:id="rId5"/>
   </sheets>
 </workbook>
 </file>
@@ -398,11 +401,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C43"/>
+  <dimension ref="A1:C34"/>
   <cols>
-    <col min="1" max="1" width="32.83203125" customWidth="1"/>
+    <col min="1" max="1" width="56.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
-    <col min="3" max="3" width="22.83203125" customWidth="1"/>
+    <col min="3" max="3" width="38.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -418,7 +421,7 @@
         <v/>
       </c>
       <c r="C3" t="str">
-        <v>Distance moyenne : 14 km</v>
+        <v>Distance moyenne : 19 km ---- Écart-type : 3</v>
       </c>
     </row>
     <row r="4">
@@ -426,7 +429,7 @@
         <v>Équipe</v>
       </c>
       <c r="B4" t="str">
-        <v>Club</v>
+        <v>Numéro Club</v>
       </c>
       <c r="C4" t="str">
         <v>Distance totale (km)</v>
@@ -434,35 +437,35 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v/>
+        <v>VALLEE BASKET CLUB-8</v>
       </c>
       <c r="B5" t="str">
-        <v/>
+        <v>PDL0049117</v>
       </c>
       <c r="C5" t="str">
-        <v>28</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v/>
+        <v>ANDARD BRAIN-2</v>
       </c>
       <c r="B6" t="str">
-        <v/>
+        <v>PDL0049004</v>
       </c>
       <c r="C6" t="str">
-        <v>28</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v/>
+        <v>CHAMP SUR LAYON USND-1</v>
       </c>
       <c r="B7" t="str">
-        <v/>
+        <v>PDL0049032</v>
       </c>
       <c r="C7" t="str">
-        <v>30</v>
+        <v>41</v>
       </c>
     </row>
     <row r="9">
@@ -473,7 +476,7 @@
         <v/>
       </c>
       <c r="C9" t="str">
-        <v>Distance moyenne : 9 km</v>
+        <v>Distance moyenne : 9 km ---- Écart-type : 3</v>
       </c>
     </row>
     <row r="10">
@@ -481,7 +484,7 @@
         <v>Équipe</v>
       </c>
       <c r="B10" t="str">
-        <v>Club</v>
+        <v>Numéro Club</v>
       </c>
       <c r="C10" t="str">
         <v>Distance totale (km)</v>
@@ -489,322 +492,308 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v/>
+        <v>SAINT CHRISTOPHE DU BOIS - ESSOR CHRISTOPHORIEN BASKET-1</v>
       </c>
       <c r="B11" t="str">
-        <v/>
+        <v>PDL0049097</v>
       </c>
       <c r="C11" t="str">
-        <v>14</v>
+        <v>29</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v/>
+        <v>PUY SAINT BONNET BASKET-1</v>
       </c>
       <c r="B12" t="str">
-        <v/>
+        <v>PDL0049093</v>
       </c>
       <c r="C12" t="str">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v/>
+        <v>LA TESSOUALLE-1</v>
       </c>
       <c r="B13" t="str">
-        <v/>
+        <v>PDL0049124</v>
       </c>
       <c r="C13" t="str">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>Poule C</v>
-      </c>
-      <c r="B15" t="str">
-        <v/>
-      </c>
-      <c r="C15" t="str">
-        <v>Distance moyenne : 21 km</v>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>MAULEVRIER-1</v>
+      </c>
+      <c r="B14" t="str">
+        <v>PDL0049074</v>
+      </c>
+      <c r="C14" t="str">
+        <v>34</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Équipe</v>
+        <v>Poule C</v>
       </c>
       <c r="B16" t="str">
-        <v>Club</v>
+        <v/>
       </c>
       <c r="C16" t="str">
-        <v>Distance totale (km)</v>
+        <v>Distance moyenne : 21 km ---- Écart-type : 3</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v/>
+        <v>Équipe</v>
       </c>
       <c r="B17" t="str">
-        <v/>
+        <v>Numéro Club</v>
       </c>
       <c r="C17" t="str">
-        <v>52</v>
+        <v>Distance totale (km)</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v/>
+        <v>ESSJ GREZ NEUVILLE-1</v>
       </c>
       <c r="B18" t="str">
-        <v/>
+        <v>PDL0049061</v>
       </c>
       <c r="C18" t="str">
-        <v>39</v>
+        <v>52</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v/>
+        <v>ELAN LIGÉRIEN BASKET-2</v>
       </c>
       <c r="B19" t="str">
-        <v/>
+        <v>PDL0049115</v>
       </c>
       <c r="C19" t="str">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>SAINTE GEMMES SUR LOIRE-1</v>
+      </c>
+      <c r="B20" t="str">
+        <v>PDL0049143</v>
+      </c>
+      <c r="C20" t="str">
         <v>36</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="str">
-        <v>Poule D</v>
-      </c>
-      <c r="B21" t="str">
-        <v/>
-      </c>
-      <c r="C21" t="str">
-        <v>Distance moyenne : 7 km</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Équipe</v>
+        <v>Poule D</v>
       </c>
       <c r="B22" t="str">
-        <v>Club</v>
+        <v/>
       </c>
       <c r="C22" t="str">
-        <v>Distance totale (km)</v>
+        <v>Distance moyenne : 14 km ---- Écart-type : 2</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v/>
+        <v>Équipe</v>
       </c>
       <c r="B23" t="str">
-        <v/>
+        <v>Numéro Club</v>
       </c>
       <c r="C23" t="str">
-        <v>19</v>
+        <v>Distance totale (km)</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v/>
+        <v>VAL HYROME BASKET-1</v>
       </c>
       <c r="B24" t="str">
-        <v/>
+        <v>PDL0049027</v>
       </c>
       <c r="C24" t="str">
-        <v>11</v>
+        <v>46</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v/>
+        <v>CORON/SALLE DE VIHIERS-1</v>
       </c>
       <c r="B25" t="str">
-        <v/>
+        <v>PDL0049050</v>
       </c>
       <c r="C25" t="str">
-        <v>12</v>
+        <v>49</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>BASKET LA GAULOISE LA CHAPELLE ROUSSELIN-1</v>
+      </c>
+      <c r="B26" t="str">
+        <v>PDL0049036</v>
+      </c>
+      <c r="C26" t="str">
+        <v>33</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Poule E</v>
+        <v>JUB JALLAIS BASKET-1</v>
       </c>
       <c r="B27" t="str">
-        <v/>
+        <v>PDL0049063</v>
       </c>
       <c r="C27" t="str">
-        <v>Distance moyenne : 17 km</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="str">
-        <v>Équipe</v>
-      </c>
-      <c r="B28" t="str">
-        <v>Club</v>
-      </c>
-      <c r="C28" t="str">
-        <v>Distance totale (km)</v>
+        <v>43</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v/>
+        <v>Poule E</v>
       </c>
       <c r="B29" t="str">
         <v/>
       </c>
       <c r="C29" t="str">
-        <v>38</v>
+        <v>Distance moyenne : 16 km ---- Écart-type : 5</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v/>
+        <v>Équipe</v>
       </c>
       <c r="B30" t="str">
-        <v/>
+        <v>Numéro Club</v>
       </c>
       <c r="C30" t="str">
-        <v>34</v>
+        <v>Distance totale (km)</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v/>
+        <v>POITEVINIERE LE PIN-2</v>
       </c>
       <c r="B31" t="str">
-        <v/>
+        <v>PDL0049084</v>
       </c>
       <c r="C31" t="str">
-        <v>32</v>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>CHOLET JF-1</v>
+      </c>
+      <c r="B32" t="str">
+        <v>PDL0049045</v>
+      </c>
+      <c r="C32" t="str">
+        <v>40</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Poule F</v>
+        <v>CTC ANDREA MACAIROIS BASKET​-1</v>
       </c>
       <c r="B33" t="str">
-        <v/>
+        <v>PDL0049170</v>
       </c>
       <c r="C33" t="str">
-        <v>Distance moyenne : 19 km</v>
+        <v>39</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Équipe</v>
+        <v>CHOLET BASKET-3</v>
       </c>
       <c r="B34" t="str">
-        <v>Club</v>
+        <v>PDL0049043</v>
       </c>
       <c r="C34" t="str">
-        <v>Distance totale (km)</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="str">
-        <v/>
-      </c>
-      <c r="B35" t="str">
-        <v/>
-      </c>
-      <c r="C35" t="str">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="str">
-        <v/>
-      </c>
-      <c r="B36" t="str">
-        <v/>
-      </c>
-      <c r="C36" t="str">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="str">
-        <v/>
-      </c>
-      <c r="B37" t="str">
-        <v/>
-      </c>
-      <c r="C37" t="str">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="str">
-        <v>Poule G</v>
-      </c>
-      <c r="B39" t="str">
-        <v/>
-      </c>
-      <c r="C39" t="str">
-        <v>Distance moyenne : 15 km</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="str">
-        <v>Équipe</v>
-      </c>
-      <c r="B40" t="str">
-        <v>Club</v>
-      </c>
-      <c r="C40" t="str">
-        <v>Distance totale (km)</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="str">
-        <v/>
-      </c>
-      <c r="B41" t="str">
-        <v/>
-      </c>
-      <c r="C41" t="str">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="str">
-        <v/>
-      </c>
-      <c r="B42" t="str">
-        <v/>
-      </c>
-      <c r="C42" t="str">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="str">
-        <v/>
-      </c>
-      <c r="B43" t="str">
-        <v/>
-      </c>
-      <c r="C43" t="str">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C43"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C34"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1"/>
+  <cols>
+    <col min="1" max="1" width="56.83203125" customWidth="1"/>
+    <col min="2" max="2" width="20.83203125" customWidth="1"/>
+    <col min="3" max="3" width="38.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>SENIOR — masculin — Niveau 2</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1"/>
+  <cols>
+    <col min="1" max="1" width="56.83203125" customWidth="1"/>
+    <col min="2" max="2" width="20.83203125" customWidth="1"/>
+    <col min="3" max="3" width="38.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>SENIOR — masculin — Niveau 3</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1"/>
+  <cols>
+    <col min="1" max="1" width="56.83203125" customWidth="1"/>
+    <col min="2" max="2" width="20.83203125" customWidth="1"/>
+    <col min="3" max="3" width="38.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>SENIOR — masculin — Niveau 4</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:G7"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -848,27 +837,96 @@
         <v>Niveau 1</v>
       </c>
       <c r="B4">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C4">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D4" t="str">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E4" t="str">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F4" t="str">
         <v>21</v>
       </c>
       <c r="G4" t="str">
-        <v>14</v>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Niveau 2</v>
+      </c>
+      <c r="B5">
+        <v>0</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5" t="str">
+        <v>0</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Infinity</v>
+      </c>
+      <c r="F5" t="str">
+        <v>-Infinity</v>
+      </c>
+      <c r="G5" t="str">
+        <v>-Infinity</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Niveau 3</v>
+      </c>
+      <c r="B6">
+        <v>0</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+      <c r="D6" t="str">
+        <v>0</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Infinity</v>
+      </c>
+      <c r="F6" t="str">
+        <v>-Infinity</v>
+      </c>
+      <c r="G6" t="str">
+        <v>-Infinity</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Niveau 4</v>
+      </c>
+      <c r="B7">
+        <v>0</v>
+      </c>
+      <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="D7" t="str">
+        <v>0</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Infinity</v>
+      </c>
+      <c r="F7" t="str">
+        <v>-Infinity</v>
+      </c>
+      <c r="G7" t="str">
+        <v>-Infinity</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>